<commit_message>
feat(examples): replace toy data with 500-student 10-item standard IRT 3PL dataset
</commit_message>
<xml_diff>
--- a/examples/sample_answers.xlsx
+++ b/examples/sample_answers.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -382,7 +382,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -402,7 +402,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -412,7 +412,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>程序執行</t>
+          <t>概念理解</t>
         </is>
       </c>
     </row>
@@ -422,7 +422,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -432,7 +432,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>解題思考</t>
+          <t>程序執行</t>
         </is>
       </c>
     </row>
@@ -442,7 +442,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -462,17 +462,117 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>數與計算</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>程序執行</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>數與計算</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>程序執行</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>空間與形狀</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>概念理解</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>數與計算</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>概念理解</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>關係</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>概念理解</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>數與計算</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>解題思考</t>
         </is>
       </c>
     </row>

</xml_diff>